<commit_message>
Add problem handle when the X cannot be open/ cannot be scraped.
</commit_message>
<xml_diff>
--- a/TestAccount.xlsx
+++ b/TestAccount.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chenzhijun/GithubProject/Twitter-Scraper-Script/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3712092-3B01-7644-B010-ED83C872E283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B528A904-7D88-3444-AA91-F950367F4C5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="960" windowWidth="27640" windowHeight="15840" xr2:uid="{EEF32252-7FA9-244D-B505-6931E17D627F}"/>
   </bookViews>
@@ -36,18 +36,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>username</t>
   </si>
   <si>
     <t>password</t>
-  </si>
-  <si>
-    <t>@chengxihan1</t>
-  </si>
-  <si>
-    <t>Shuaijerryshuai2448878048</t>
   </si>
   <si>
     <t>@MaxSun19455616</t>
@@ -431,7 +425,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4374B3B0-9476-304A-9B67-771E911E4A0C}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -444,26 +438,18 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert "Add problem handle when the X cannot be open/ cannot be scraped."
This reverts commit 430ed6f6eb2087ca0dc92156ef81a0270af07a54.
</commit_message>
<xml_diff>
--- a/TestAccount.xlsx
+++ b/TestAccount.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chenzhijun/GithubProject/Twitter-Scraper-Script/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B528A904-7D88-3444-AA91-F950367F4C5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3712092-3B01-7644-B010-ED83C872E283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="960" windowWidth="27640" windowHeight="15840" xr2:uid="{EEF32252-7FA9-244D-B505-6931E17D627F}"/>
   </bookViews>
@@ -36,12 +36,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>username</t>
   </si>
   <si>
     <t>password</t>
+  </si>
+  <si>
+    <t>@chengxihan1</t>
+  </si>
+  <si>
+    <t>Shuaijerryshuai2448878048</t>
   </si>
   <si>
     <t>@MaxSun19455616</t>
@@ -425,7 +431,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4374B3B0-9476-304A-9B67-771E911E4A0C}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -438,18 +444,26 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>